<commit_message>
plan tesis to review
</commit_message>
<xml_diff>
--- a/anexos/Matriz_Consistencia_Grupo9.2.xlsx
+++ b/anexos/Matriz_Consistencia_Grupo9.2.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -498,330 +498,338 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Problema general: ¿En qué medida un contrato OpenAPI bancario se alinea con el modelo de referencia BIAN y bajo qué tipologías se produce desalineación?</t>
+          <t>Problema tecnológico: No existe un método reproducible que cuantifique en qué medida un contrato OpenAPI bancario se alinea con un Service Domain BIAN y bajo qué tipologías se desalinea.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Objetivo general: Diseñar y aplicar un modelo de alineación que calcule SemanticScore (S), StructuralScore (E), CoverageScore (C) y un AlignmentScore integrado para evaluar contratos OpenAPI frente a Service Domains BIAN.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+          <t>Objetivo general (técnico): Diseñar un modelo de alineación y el procedimiento que calculen SemanticScore (S), StructuralScore (E), CoverageScore (C) y AlignmentScore integrado para evaluar contratos OpenAPI frente a Service Domains BIAN (Guía 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Objetivo superior: Si el artefacto existiera: equipos de arquitectura/API podrían cuantificar la coherencia OpenAPI–BIAN antes del despliegue, reduciendo retrabajo en integraciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Fase</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Problema</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Objetivo</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Producto verificable</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Variable Independiente</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Estados de la Variable Independiente</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>Variable Dependiente</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Estados del factor</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Ratio (resultado)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Hipótesis</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Indicadores / Métricas de la Variable Dependiente</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Variables de Control</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Fase 1 — Diseño del modelo de alineación</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Marco metodológico: no existe un modelo documentado para cuantificar la alineación entre contratos OpenAPI bancarios y Service Domains BIAN (no confundir con P1).</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Diseñar el modelo de alineación OpenAPI ↔ BIAN, definiendo entradas, componentes de score (S, E, C), fórmula de agregación y criterios de clasificación.</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Modelo metodológico documentado: adquisición → normalización → SemanticScore (S) + StructuralScore (E) + CoverageScore (C) → AlignmentScore.</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>No aplica</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>No aplica</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Adecuación del diseño del modelo</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Un modelo estructurado por componentes S, E y C permite calcular de forma reproducible un score de alineación interpretable entre OpenAPI y BIAN.</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Cobertura del modelo (nº de etapas y scores definidos), trazabilidad entrada→salida, criterios de validez explícitos.</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Ámbito: sector bancario; contratos OpenAPI 3.x evaluados contra Service Domains BIAN; alcance documental (sin despliegue en producción).</t>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Indicadores / Métricas del ratio</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Parámetros de control</t>
         </is>
       </c>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Fase 2 — Adquisición y normalización de artefactos (OE1)</t>
+          <t>Fase 1 — Diseño del modelo de alineación</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Los contratos OpenAPI bancarios y los Service Domains BIAN expresan el dominio en vistas conceptuales distintas (REST vs. negocio), lo que impide compararlos directamente (P1, P2).</t>
+          <t>Problema tecnológico (Fase 1): no existe un método reproducible que cuantifique en qué medida un contrato OpenAPI bancario se alinea con un Service Domain BIAN y bajo qué tipologías se desalinea (distinto de la problemática del sector, §1.2).</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Transformar contratos OpenAPI y artefactos BIAN en representaciones normalizadas y comparables sobre un modelo intermedio común.</t>
+          <t>Diseñar el modelo de alineación OpenAPI ↔ BIAN, definiendo entradas, componentes de score (S, E, C), fórmula de agregación y criterios de clasificación.</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Conjunto de representaciones normalizadas versionadas (paths, operations, schemas, behaviors, business objects) listas para el cálculo de scores.</t>
+          <t>Modelo metodológico documentado: adquisición → normalización → SemanticScore (S) + StructuralScore (E) + CoverageScore (C) → AlignmentScore.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Esquema de representación intermedia</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Modelo tabular (recurso–operación–esquema); modelo en grafo (nodos/aristas); modelo RDF/triples (opcional).</t>
+          <t>No aplica</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Calidad y completitud de la extracción estructural</t>
+          <t>Adecuación del diseño del modelo</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>La normalización de OpenAPI bancario y BIAN en un modelo intermedio común habilita el cálculo sistemático de los scores S, E y C.</t>
+          <t>Un modelo estructurado por componentes S, E y C permite calcular de forma reproducible un score de alineación interpretable entre OpenAPI y BIAN.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>Nº de elementos extraídos (endpoints, schemas, behaviors, business objects); % de cobertura respecto al artefacto fuente; integridad de metadatos.</t>
+          <t>Cobertura del modelo (nº de etapas y scores definidos), trazabilidad entrada→salida, criterios de validez explícitos.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Versión fija del contrato OpenAPI y del Service Domain BIAN emparejados; herramientas de parsing fijas; mismo ámbito sectorial.</t>
+          <t>Ámbito: sector bancario; contratos OpenAPI 3.x evaluados contra Service Domains BIAN; alcance documental (sin despliegue en producción).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Fase 3 — Cálculo del StructuralScore E (OE2 · P1)</t>
+          <t>Fase 2 — Adquisición y normalización de artefactos (OE1)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>No se conocen las correspondencias de jerarquía y organización entre endpoints, recursos y esquemas OpenAPI y los elementos del Service Domain BIAN.</t>
+          <t>Los contratos OpenAPI bancarios y los Service Domains BIAN expresan el dominio en vistas conceptuales distintas (REST vs. negocio), lo que impide compararlos directamente (P1, P2).</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Calcular el StructuralScore (E): correspondencia estructural entre componentes OpenAPI y artefactos BIAN normalizados.</t>
+          <t>Transformar contratos OpenAPI y artefactos BIAN en representaciones normalizadas y comparables sobre un modelo intermedio común.</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Matriz de correspondencias estructurales y StructuralScore (E) normalizado [0, 1].</t>
+          <t>Conjunto de representaciones normalizadas versionadas (paths, operations, schemas, behaviors, business objects) listas para el cálculo de scores.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Estrategia de matching estructural (schema matching)</t>
+          <t>Esquema de representación intermedia</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Correspondencia por nombre exacto; similitud de ruta/recurso; correspondencia por profundidad y tipo de esquema; matching por operación HTTP.</t>
+          <t>Modelo tabular (recurso–operación–esquema); modelo en grafo (nodos/aristas); modelo RDF/triples (opcional).</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>StructuralScore (E) — alineación estructural OpenAPI ↔ BIAN</t>
+          <t>Calidad y completitud de la extracción estructural</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Las técnicas de schema matching producen un StructuralScore que refleja la correspondencia entre la organización REST y el modelo BIAN.</t>
+          <t>La normalización de OpenAPI bancario y BIAN en un modelo intermedio común habilita el cálculo sistemático de los scores S, E y C.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>StructuralScore E ∈ [0, 1]; tasa de correspondencia estructural (%); nº de pares alineados; desalineaciones estructurales detectadas.</t>
+          <t>Nº de elementos extraídos (endpoints, schemas, behaviors, business objects); % de cobertura respecto al artefacto fuente; integridad de metadatos.</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Mismo conjunto normalizado de la Fase 2; umbral de correspondencia fijo; sin intervención manual en el matching.</t>
+          <t>Versión fija del contrato OpenAPI y del Service Domain BIAN emparejados; herramientas de parsing fijas; mismo ámbito sectorial.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Fase 4 — Cálculo del SemanticScore S (OE3 · P2)</t>
+          <t>Fase 3 — Cálculo del StructuralScore E (OE2 · P1)</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Se desconoce el grado de equivalencia semántica entre términos de negocio BIAN y nombres/descripciones en contratos OpenAPI bancarios.</t>
+          <t>No se conocen las correspondencias de jerarquía y organización entre endpoints, recursos y esquemas OpenAPI y los elementos del Service Domain BIAN.</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Calcular el SemanticScore (S): similitud semántica entre conceptos de negocio BIAN y componentes del contrato OpenAPI.</t>
+          <t>Calcular el StructuralScore (E): correspondencia estructural entre componentes OpenAPI y artefactos BIAN normalizados.</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Matriz de similitud semántica y SemanticScore (S) normalizado [0, 1].</t>
+          <t>Matriz de correspondencias estructurales y StructuralScore (E) normalizado [0, 1].</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Técnica de similitud semántica</t>
+          <t>Estrategia de matching estructural (schema matching)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Embeddings + similitud coseno; matching léxico/ontológico; enfoque híbrido (estructural + semántico).</t>
+          <t>Correspondencia por nombre exacto; similitud de ruta/recurso; correspondencia por profundidad y tipo de esquema; matching por operación HTTP.</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>SemanticScore (S) — alineación semántica OpenAPI ↔ BIAN</t>
+          <t>StructuralScore (E) — alineación estructural OpenAPI ↔ BIAN</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Las métricas de similitud semántica producen un SemanticScore que discrimina conceptos alineados de desalineaciones semánticas o de modelado.</t>
+          <t>Las técnicas de schema matching producen un StructuralScore que refleja la correspondencia entre la organización REST y el modelo BIAN.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>SemanticScore S ∈ [0, 1]; similitud coseno promedio; nº de pares sobre umbral; distribución por tipología (semántica, modelado).</t>
+          <t>StructuralScore E ∈ [0, 1]; tasa de correspondencia estructural (%); nº de pares alineados; desalineaciones estructurales detectadas.</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Mismo corpus de términos; umbral de similitud fijo; misma técnica de embedding/modelo por corrida.</t>
+          <t>Mismo conjunto normalizado de la Fase 2; umbral de correspondencia fijo; sin intervención manual en el matching.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>Fase 4 — Cálculo del SemanticScore S (OE3 · P2)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Se desconoce el grado de equivalencia semántica entre términos de negocio BIAN y nombres/descripciones en contratos OpenAPI bancarios.</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Calcular el SemanticScore (S): similitud semántica entre conceptos de negocio BIAN y componentes del contrato OpenAPI.</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Matriz de similitud semántica y SemanticScore (S) normalizado [0, 1].</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Técnica de similitud semántica</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Embeddings + similitud coseno; matching léxico/ontológico; enfoque híbrido (estructural + semántico).</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>SemanticScore (S) — alineación semántica OpenAPI ↔ BIAN</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Las métricas de similitud semántica producen un SemanticScore que discrimina conceptos alineados de desalineaciones semánticas o de modelado.</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>SemanticScore S ∈ [0, 1]; similitud coseno promedio; nº de pares sobre umbral; distribución por tipología (semántica, modelado).</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>Mismo corpus de términos; umbral de similitud fijo; misma técnica de embedding/modelo por corrida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
           <t>Fase 5 — CoverageScore, AlignmentScore y clasificación (OE4 · P3–P4)</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>No existe un indicador integrado que combine alineación semántica, estructural y cobertura de conceptos BIAN, ni una escala interpretable de alineación global.</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Calcular CoverageScore (C), obtener AlignmentScore = α·S + β·E + γ·C (α + β + γ = 1) y clasificar el nivel de alineación del contrato OpenAPI.</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>CoverageScore (C); AlignmentScore; clasificación (Alta ≥0,80 · Media 0,60–0,79 · Baja 0,40–0,59 · Nula &lt;0,40); informe de tipologías de desalineación.</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Pesos de agregación (α, β, γ)</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Pesos iguales (α=β=γ=1/3); ponderación experta; sensibilidad por tipología dominante.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>AlignmentScore — alineación global OpenAPI ↔ BIAN</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>La agregación ponderada de S, E y C produce un AlignmentScore interpretable y clasificable por niveles de alineación del contrato OpenAPI bancario.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>CoverageScore C ∈ [0, 1]; AlignmentScore = α·S + β·E + γ·C; nivel de alineación (Alta/Media/Baja/Nula); frecuencia por tipología (estructural, semántica, modelado, REST/contrato).</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Pesos α + β + γ = 1 fijos por corrida; mismos S, E, C de Fases 3–4; misma taxonomía de desalineaciones (Tabla 2, Cap. 1); umbrales de clasificación fijos.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A5:J5"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A2:J2"/>
@@ -837,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -865,199 +873,199 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Problema general</t>
+          <t>Problemática (situación real)</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>¿En qué medida un contrato OpenAPI bancario se alinea con el modelo de referencia BIAN y bajo qué tipologías se produce desalineación?</t>
+          <t>Síntomas sector bancario — §1.2</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Cap. 1 §1.3</t>
+          <t>Cap. 1 §1.2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Objetivo general</t>
+          <t>Problema abstracto</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Diseñar y aplicar un modelo de alineación que calcule SemanticScore (S), StructuralScore (E), CoverageScore (C) y un AlignmentScore integrado para evaluar contratos OpenAPI frente a Service Domains BIAN.</t>
+          <t>Correspondencia OpenAPI ↔ BIAN — §1.3</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Cap. 2 §2.2</t>
+          <t>Cap. 1 §1.3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>OE1</t>
+          <t>Problema tecnológico</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Transformar contratos OpenAPI y artefactos BIAN en representaciones normalizadas y comparables sobre un modelo intermedio común.</t>
+          <t>No existe un método reproducible que cuantifique en qué medida un contrato OpenAPI bancario se alinea con un Service Domain BIAN y bajo qué tipologías se desalinea.</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Fase 2 — Normalización</t>
+          <t>Cap. 1 §1.3 · Anexo C</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>OE2</t>
+          <t>Objetivo superior</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Calcular el StructuralScore (E): correspondencia estructural entre componentes OpenAPI y artefactos BIAN normalizados.</t>
+          <t>Si el artefacto existiera: equipos de arquitectura/API podrían cuantificar la coherencia OpenAPI–BIAN antes del despliegue, reduciendo retrabajo en integraciones.</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Fase 3 — StructuralScore (E)</t>
+          <t>Cap. 2 §2.2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>OE3</t>
+          <t>Objetivo general (técnico)</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Calcular el SemanticScore (S): similitud semántica entre conceptos de negocio BIAN y componentes del contrato OpenAPI.</t>
+          <t>Diseñar un modelo de alineación y el procedimiento que calculen SemanticScore (S), StructuralScore (E), CoverageScore (C) y AlignmentScore integrado para evaluar contratos OpenAPI frente a Service Domains BIAN (Guía 1).</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Fase 4 — SemanticScore (S)</t>
+          <t>Cap. 2 §2.3</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>OE4</t>
+          <t>OE1</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Calcular CoverageScore (C), obtener AlignmentScore = α·S + β·E + γ·C (α + β + γ = 1) y clasificar el nivel de alineación del contrato OpenAPI.</t>
+          <t>Transformar contratos OpenAPI y artefactos BIAN en representaciones normalizadas y comparables sobre un modelo intermedio común.</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Fase 5 — CoverageScore + AlignmentScore</t>
+          <t>Fase 2 — Normalización</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>OE2</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Correspondencia estructural → E</t>
+          <t>Calcular el StructuralScore (E): correspondencia estructural entre componentes OpenAPI y artefactos BIAN normalizados.</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 3 — StructuralScore (E)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>OE3</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Similitud semántica → S</t>
+          <t>Calcular el SemanticScore (S): similitud semántica entre conceptos de negocio BIAN y componentes del contrato OpenAPI.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 4 — SemanticScore (S)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>P3–P4</t>
+          <t>OE4</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Cobertura + score global → C + AlignmentScore</t>
+          <t>Calcular CoverageScore (C), obtener AlignmentScore = α·S + β·E + γ·C (α + β + γ = 1) y clasificar el nivel de alineación del contrato OpenAPI.</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Fase 5</t>
+          <t>Fase 5 — CoverageScore + AlignmentScore</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>SemanticScore (S)</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Similitud de significado OpenAPI ↔ BIAN</t>
+          <t>Correspondencia estructural → E</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>StructuralScore (E)</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Correspondencia de jerarquía y organización</t>
+          <t>Similitud semántica → S</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>CoverageScore (C)</t>
+          <t>P3–P4</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Conceptos BIAN cubiertos por el contrato</t>
+          <t>Cobertura + score global → C + AlignmentScore</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -1069,15 +1077,66 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
+          <t>SemanticScore (S)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Similitud de significado OpenAPI ↔ BIAN</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Fase 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>StructuralScore (E)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Correspondencia de jerarquía y organización</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Fase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>CoverageScore (C)</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Conceptos BIAN cubiertos por el contrato</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Fase 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>AlignmentScore</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>α·S + β·E + γ·C (α+β+γ=1); clasificación Alta/Media/Baja/Nula</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Fase 5 · Anexo figuras_alineacion_openapi_bian.pdf</t>
         </is>

</xml_diff>